<commit_message>
P8: update 9 files
</commit_message>
<xml_diff>
--- a/packages/central-server/exported-refdata-all-table.xlsx
+++ b/packages/central-server/exported-refdata-all-table.xlsx
@@ -445,22 +445,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>923f5b09-3229-4bda-9a40-576f887faca2</v>
+        <v>1ed6a4ae-ca3a-4aba-8c8f-01a4e632f3c4</v>
       </c>
       <c r="B2" t="str">
-        <v>BEJS092256</v>
+        <v>OSUC515697</v>
       </c>
       <c r="C2" t="str">
-        <v>Walter</v>
+        <v>David</v>
       </c>
       <c r="E2" t="str">
-        <v>Piccioli</v>
+        <v>Bucelli</v>
       </c>
       <c r="F2" t="str">
-        <v>Rhodes</v>
+        <v>Bos</v>
       </c>
       <c r="G2" s="1">
-        <v>28973</v>
+        <v>29915</v>
       </c>
       <c r="I2" t="str">
         <v>male</v>

</xml_diff>

<commit_message>
workhorse/u6:TAM-6886: Sensitive networks project
</commit_message>
<xml_diff>
--- a/packages/central-server/exported-refdata-all-table.xlsx
+++ b/packages/central-server/exported-refdata-all-table.xlsx
@@ -445,22 +445,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1ed6a4ae-ca3a-4aba-8c8f-01a4e632f3c4</v>
+        <v>64ab6957-2932-4766-9f5c-a58a90e01aef</v>
       </c>
       <c r="B2" t="str">
-        <v>OSUC515697</v>
+        <v>YGLR199428</v>
       </c>
       <c r="C2" t="str">
-        <v>David</v>
+        <v>Bernard</v>
       </c>
       <c r="E2" t="str">
-        <v>Bucelli</v>
+        <v>Lippi</v>
       </c>
       <c r="F2" t="str">
-        <v>Bos</v>
+        <v>Gensini</v>
       </c>
       <c r="G2" s="1">
-        <v>29915</v>
+        <v>28860</v>
       </c>
       <c r="I2" t="str">
         <v>male</v>

</xml_diff>